<commit_message>
Separate account of Twilio and ElevenLabs
</commit_message>
<xml_diff>
--- a/resultant_excel.xlsx
+++ b/resultant_excel.xlsx
@@ -502,7 +502,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -511,7 +511,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bob Smith</t>
+          <t>Anand Swarup</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>bob.smith@example.com</t>
+          <t>anand_swarup@technologymindz.com</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>no-answer</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -564,19 +564,19 @@
           <t>"nan
 [2025-08-23 13:05:56] The customer, Bob Smith, is from the Automobile industry and wants to know how Technology Mindz can help him grow his company. The agent explains the services offered by Technology Mindz, including Salesforce implementation, robotic process automation, AI and data analytics, and cybersecurity solutions. The customer schedules a meeting with the agent for the next day at 5 p.m.
 [2025-08-23 13:22:09] No summary available. Conversation transcript missing."
-[2025-09-09 17:18:56] No summary available. Conversation transcript missing.</t>
+[2025-09-11 11:20:44] The user wants to schedule a meeting with the assistant for the next day at 5 p.m. and have a meeting invitation sent to their email.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>nan
-[2025-09-09 17:18:56] No tasks found for this call.</t>
+[2025-09-11 11:20:44] 1. Schedule a meeting, 2. Send a meeting invitation to the user's email</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7878994162</t>
+          <t>8107061392</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -635,12 +635,14 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>nan
+[2025-09-11 11:21:18] The agent introduced themselves and asked if it's a good time to talk to Vinayak from the Healthcare industry.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t xml:space="preserve">nan
+[2025-09-11 11:21:18] </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Database Athentication, New prompt feature implementation
</commit_message>
<xml_diff>
--- a/resultant_excel.xlsx
+++ b/resultant_excel.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,7 +502,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -561,88 +561,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>"nan
-[2025-08-23 13:05:56] The customer, Bob Smith, is from the Automobile industry and wants to know how Technology Mindz can help him grow his company. The agent explains the services offered by Technology Mindz, including Salesforce implementation, robotic process automation, AI and data analytics, and cybersecurity solutions. The customer schedules a meeting with the agent for the next day at 5 p.m.
-[2025-08-23 13:22:09] No summary available. Conversation transcript missing."
-[2025-09-11 11:20:44] The user wants to schedule a meeting with the assistant for the next day at 5 p.m. and have a meeting invitation sent to their email.</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>nan
-[2025-09-11 11:20:44] 1. Schedule a meeting, 2. Send a meeting invitation to the user's email</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>54</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Vinayak</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>8107061392</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>alice.johnson@example.com</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
           <t>nan</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>D Company</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Texas, USA</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>nan
-[2025-09-11 11:21:18] The agent introduced themselves and asked if it's a good time to talk to Vinayak from the Healthcare industry.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nan
-[2025-09-11 11:21:18] </t>
         </is>
       </c>
     </row>

</xml_diff>